<commit_message>
scan: seg7 2026-09-14 18:02 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-09-14.xlsx
+++ b/output/full_scan/batch_seq8_2026-09-14.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O127"/>
+  <dimension ref="A1:O128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2912,21 +2912,21 @@
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>7610</v>
+        <v>7772</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>聯友金屬-創</t>
+          <t>耀穎</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>370.5752593268726</v>
+        <v>376.5496006439943</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>1780</v>
+        <v>126</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,13 +2937,13 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>49.6821491502469</v>
+        <v>66.03180026922112</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>17.94449680482246</v>
+        <v>32.58675190006451</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>1.210499733022397</v>
+        <v>0.7495406499941943</v>
       </c>
       <c r="K47" s="2" t="n">
         <v>0</v>
@@ -2955,31 +2955,31 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>35.15536969323038</v>
+        <v>4.47290377658709</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>rsi_strong, market_above_ma60, adx_trending, stronger_than_market, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>6965</v>
+        <v>7610</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>中傑-KY</t>
+          <t>聯友金屬-創</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>363.1641965450757</v>
+        <v>370.5752593268726</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>68.59999999999999</v>
+        <v>1780</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,13 +2990,13 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>24.17388191237571</v>
+        <v>49.6821491502469</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>38.68484560137993</v>
+        <v>17.94449680482246</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>2.716419654507567</v>
+        <v>1.210499733022397</v>
       </c>
       <c r="K48" s="2" t="n">
         <v>0</v>
@@ -3008,31 +3008,31 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.4374191544628916</v>
+        <v>35.15536969323038</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>7717</v>
+        <v>6965</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>萊德光電-KY</t>
+          <t>中傑-KY</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>362.5964385728425</v>
+        <v>363.1641965450757</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>487</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,13 +3043,13 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>56.58432024180804</v>
+        <v>24.17388191237571</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>12.5554253931071</v>
+        <v>38.68484560137993</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>3.406053799562129</v>
+        <v>2.716419654507567</v>
       </c>
       <c r="K49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>9.453874353659836</v>
+        <v>-0.4374191544628916</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>8028</v>
+        <v>7717</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>昇陽半導體</t>
+          <t>萊德光電-KY</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>361.0727122861094</v>
+        <v>362.5964385728425</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>221.5</v>
+        <v>487</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,13 +3096,13 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>35.4314677661952</v>
+        <v>56.58432024180804</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>21.38144999518755</v>
+        <v>12.5554253931071</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.8854785508966629</v>
+        <v>3.406053799562129</v>
       </c>
       <c r="K50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.8146660009638786</v>
+        <v>9.453874353659836</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>volume_break, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>6922</v>
+        <v>8028</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>宸曜</t>
+          <t>昇陽半導體</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>360.9602190656016</v>
+        <v>361.0727122861094</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>185.5</v>
+        <v>221.5</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,13 +3149,13 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>41.15369513779796</v>
+        <v>35.4314677661952</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>21.93039990906952</v>
+        <v>21.38144999518755</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.28831725850119</v>
+        <v>0.8854785508966629</v>
       </c>
       <c r="K51" s="2" t="n">
         <v>0</v>
@@ -3167,31 +3167,31 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-3.101936953074741</v>
+        <v>-0.8146660009638786</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>7738</v>
+        <v>6922</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>東聯互動</t>
+          <t>宸曜</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>355.473220577063</v>
+        <v>360.9602190656016</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>163.5</v>
+        <v>185.5</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,16 +3202,16 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>38.95610487616817</v>
+        <v>41.15369513779796</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>28.95448370849522</v>
+        <v>21.93039990906952</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>0.7473220577062997</v>
+        <v>0.28831725850119</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L52" s="2" t="n">
         <v>0</v>
@@ -3220,31 +3220,31 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.8246198728063323</v>
+        <v>-3.101936953074741</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>6916</v>
+        <v>7738</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>華凌</t>
+          <t>東聯互動</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>350.0923494470436</v>
+        <v>355.473220577063</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>18.15</v>
+        <v>163.5</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,16 +3255,16 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>42.00259466446285</v>
+        <v>38.95610487616817</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>14.45350665422828</v>
+        <v>28.95448370849522</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.9220941126135096</v>
+        <v>0.7473220577062997</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.0088724010735274</v>
+        <v>-0.8246198728063323</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>6863</v>
+        <v>6916</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>永道-KY</t>
+          <t>華凌</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>348.7077657741604</v>
+        <v>350.0923494470436</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>92.90000000000001</v>
+        <v>18.15</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,13 +3308,13 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>27.20766056073574</v>
+        <v>42.00259466446285</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>21.93636377906281</v>
+        <v>14.45350665422828</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>1.15710003109925</v>
+        <v>0.9220941126135096</v>
       </c>
       <c r="K54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>-1.688813185901056</v>
+        <v>0.0088724010735274</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>7556</v>
+        <v>6863</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>意德士</t>
+          <t>永道-KY</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>348.6559672371499</v>
+        <v>348.7077657741604</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>242</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>47.37799007272434</v>
+        <v>27.20766056073574</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>23.43724184186569</v>
+        <v>21.93636377906281</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>0.3237202555917564</v>
+        <v>1.15710003109925</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-1.362267358340907</v>
+        <v>-1.688813185901056</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6951</v>
+        <v>7556</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>青新-創</t>
+          <t>意德士</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>347.5296751644131</v>
+        <v>348.6559672371499</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>69.90000000000001</v>
+        <v>242</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>31.16313354608819</v>
+        <v>47.37799007272434</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>29.14413182419603</v>
+        <v>23.43724184186569</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>1.227461410908443</v>
+        <v>0.3237202555917564</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-0.0905167540307994</v>
+        <v>-1.362267358340907</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>8033</v>
+        <v>6951</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>雷虎</t>
+          <t>青新-創</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>341.5407674411315</v>
+        <v>347.5296751644131</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>174</v>
+        <v>69.90000000000001</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,13 +3467,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>44.8619867359948</v>
+        <v>31.16313354608819</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>9.286676747359641</v>
+        <v>29.14413182419603</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.5433389717035123</v>
+        <v>1.227461410908443</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
@@ -3485,31 +3485,31 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>-1.232045088820433</v>
+        <v>-0.0905167540307994</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>6913</v>
+        <v>8033</v>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>鴻呈</t>
+          <t>雷虎</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>330.2451069738968</v>
+        <v>341.5407674411315</v>
       </c>
       <c r="E58" s="2" t="n">
-        <v>125.5</v>
+        <v>174</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -3520,13 +3520,13 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>36.23873861689518</v>
+        <v>44.8619867359948</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>23.0403983142753</v>
+        <v>9.286676747359641</v>
       </c>
       <c r="J58" s="2" t="n">
-        <v>0.5474346765615443</v>
+        <v>0.5433389717035123</v>
       </c>
       <c r="K58" s="2" t="n">
         <v>0</v>
@@ -3538,31 +3538,31 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-3.733776166695089</v>
+        <v>-1.232045088820433</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>7704</v>
+        <v>6913</v>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>明遠精密</t>
+          <t>鴻呈</t>
         </is>
       </c>
       <c r="C59" s="2" t="n">
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>328.1793348559269</v>
+        <v>330.2451069738968</v>
       </c>
       <c r="E59" s="2" t="n">
-        <v>61</v>
+        <v>125.5</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -3573,13 +3573,13 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>49.20768175502081</v>
+        <v>36.23873861689518</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>15.5001613722551</v>
+        <v>23.0403983142753</v>
       </c>
       <c r="J59" s="2" t="n">
-        <v>0.6851571464058009</v>
+        <v>0.5474346765615443</v>
       </c>
       <c r="K59" s="2" t="n">
         <v>0</v>
@@ -3591,31 +3591,31 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>-0.2469058944943223</v>
+        <v>-3.733776166695089</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>7631</v>
+        <v>7704</v>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>聚賢研發-創</t>
+          <t>明遠精密</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>326.9893362217367</v>
+        <v>328.1793348559269</v>
       </c>
       <c r="E60" s="2" t="n">
-        <v>134</v>
+        <v>61</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -3626,13 +3626,13 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>38.13313405722216</v>
+        <v>49.20768175502081</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>20.17301591441519</v>
+        <v>15.5001613722551</v>
       </c>
       <c r="J60" s="2" t="n">
-        <v>1.084299641952393</v>
+        <v>0.6851571464058009</v>
       </c>
       <c r="K60" s="2" t="n">
         <v>0</v>
@@ -3644,31 +3644,31 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-1.234852445136496</v>
+        <v>-0.2469058944943223</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>6908</v>
+        <v>7631</v>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>宏碁遊戲-創</t>
+          <t>聚賢研發-創</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>326.4528788745767</v>
+        <v>326.9893362217367</v>
       </c>
       <c r="E61" s="2" t="n">
-        <v>30.85</v>
+        <v>134</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -3679,13 +3679,13 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>45.46376965607072</v>
+        <v>38.13313405722216</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>26.56500766104792</v>
+        <v>20.17301591441519</v>
       </c>
       <c r="J61" s="2" t="n">
-        <v>0.1812327451323905</v>
+        <v>1.084299641952393</v>
       </c>
       <c r="K61" s="2" t="n">
         <v>0</v>
@@ -3697,31 +3697,31 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.2036819765576367</v>
+        <v>-1.234852445136496</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>6953</v>
+        <v>6908</v>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>家碩</t>
+          <t>宏碁遊戲-創</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>323.3259390166036</v>
+        <v>326.4528788745767</v>
       </c>
       <c r="E62" s="2" t="n">
-        <v>228</v>
+        <v>30.85</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -3732,16 +3732,16 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>46.90756100085044</v>
+        <v>45.46376965607072</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>17.31308320240028</v>
+        <v>26.56500766104792</v>
       </c>
       <c r="J62" s="2" t="n">
-        <v>0.7737137795183813</v>
+        <v>0.1812327451323905</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L62" s="2" t="n">
         <v>0</v>
@@ -3750,31 +3750,31 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-1.291408958742627</v>
+        <v>0.2036819765576367</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>7780</v>
+        <v>6953</v>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>大研生醫*</t>
+          <t>家碩</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
         <v/>
       </c>
       <c r="D63" s="2" t="n">
-        <v>322.9642246232042</v>
+        <v>323.3259390166036</v>
       </c>
       <c r="E63" s="2" t="n">
-        <v>16.1</v>
+        <v>228</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -3785,16 +3785,16 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>32.85460374897704</v>
+        <v>46.90756100085044</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>16.5076709113145</v>
+        <v>17.31308320240028</v>
       </c>
       <c r="J63" s="2" t="n">
-        <v>1.574190862705522</v>
+        <v>0.7737137795183813</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L63" s="2" t="n">
         <v>0</v>
@@ -3803,31 +3803,31 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-0.0425227082970786</v>
+        <v>-1.291408958742627</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>7751</v>
+        <v>7780</v>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>竑騰</t>
+          <t>大研生醫*</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
         <v/>
       </c>
       <c r="D64" s="2" t="n">
-        <v>321.8939367637042</v>
+        <v>322.9642246232042</v>
       </c>
       <c r="E64" s="2" t="n">
-        <v>1405</v>
+        <v>16.1</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -3838,49 +3838,49 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>44.29735165763189</v>
+        <v>32.85460374897704</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>15.0122034974085</v>
+        <v>16.5076709113145</v>
       </c>
       <c r="J64" s="2" t="n">
-        <v>0.4468394223369706</v>
+        <v>1.574190862705522</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L64" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M64" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-39.26818117507665</v>
+        <v>-0.0425227082970786</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>volume_break, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>7402</v>
+        <v>7751</v>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>邑錡</t>
+          <t>竑騰</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>318.5719225141462</v>
+        <v>321.8939367637042</v>
       </c>
       <c r="E65" s="2" t="n">
-        <v>101.5</v>
+        <v>1405</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -3891,49 +3891,49 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>42.81000961880275</v>
+        <v>44.29735165763189</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>14.97552822243574</v>
+        <v>15.0122034974085</v>
       </c>
       <c r="J65" s="2" t="n">
-        <v>0.2915232571964776</v>
+        <v>0.4468394223369706</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L65" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M65" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.7372415891195636</v>
+        <v>-39.26818117507665</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>7795</v>
+        <v>7402</v>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>長廣</t>
+          <t>邑錡</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>315.1227702096353</v>
+        <v>318.5719225141462</v>
       </c>
       <c r="E66" s="2" t="n">
-        <v>491</v>
+        <v>101.5</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -3944,13 +3944,13 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>45.61386857436201</v>
+        <v>42.81000961880275</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>17.00805359967658</v>
+        <v>14.97552822243574</v>
       </c>
       <c r="J66" s="2" t="n">
-        <v>0.9707986746994964</v>
+        <v>0.2915232571964776</v>
       </c>
       <c r="K66" s="2" t="n">
         <v>0</v>
@@ -3962,31 +3962,31 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-6.901192910045916</v>
+        <v>-0.7372415891195636</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>7768</v>
+        <v>7795</v>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>頌勝科技</t>
+          <t>長廣</t>
         </is>
       </c>
       <c r="C67" s="2" t="n">
         <v/>
       </c>
       <c r="D67" s="2" t="n">
-        <v>314.9584245658006</v>
+        <v>315.1227702096353</v>
       </c>
       <c r="E67" s="2" t="n">
-        <v>255.5</v>
+        <v>491</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -3997,13 +3997,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>35.62787852446321</v>
+        <v>45.61386857436201</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>17.81084298450024</v>
+        <v>17.00805359967658</v>
       </c>
       <c r="J67" s="2" t="n">
-        <v>0.4582627111956998</v>
+        <v>0.9707986746994964</v>
       </c>
       <c r="K67" s="2" t="n">
         <v>0</v>
@@ -4015,31 +4015,31 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-2.414957345846922</v>
+        <v>-6.901192910045916</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>7839</v>
+        <v>7768</v>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>達人網</t>
+          <t>頌勝科技</t>
         </is>
       </c>
       <c r="C68" s="2" t="n">
         <v/>
       </c>
       <c r="D68" s="2" t="n">
-        <v>313.0394793325109</v>
+        <v>314.9584245658006</v>
       </c>
       <c r="E68" s="2" t="n">
-        <v>43.35</v>
+        <v>255.5</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -4050,16 +4050,16 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>42.98115845494715</v>
+        <v>35.62787852446321</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>42.71388489358979</v>
+        <v>17.81084298450024</v>
       </c>
       <c r="J68" s="2" t="n">
-        <v>0.5206657501389417</v>
+        <v>0.4582627111956998</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L68" s="2" t="n">
         <v>0</v>
@@ -4068,31 +4068,31 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-0.1211103875528896</v>
+        <v>-2.414957345846922</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6936</v>
+        <v>7839</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>永鴻生技</t>
+          <t>達人網</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>309.3126404386568</v>
+        <v>313.0394793325109</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>31.6</v>
+        <v>43.35</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,16 +4103,16 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>36.42833219344814</v>
+        <v>42.98115845494715</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>33.41644997318242</v>
+        <v>42.71388489358979</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>0.5395905486360973</v>
+        <v>0.5206657501389417</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L69" s="2" t="n">
         <v>0</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.1172641870784377</v>
+        <v>-0.1211103875528896</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4131,21 +4131,21 @@
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6914</v>
+        <v>6936</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>阜爾運通</t>
+          <t>永鴻生技</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>306.6920692863387</v>
+        <v>309.3126404386568</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>120</v>
+        <v>31.6</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>20.28449379277681</v>
+        <v>36.42833219344814</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>41.58421132902605</v>
+        <v>33.41644997318242</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.972105217746834</v>
+        <v>0.5395905486360973</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.3552812119583315</v>
+        <v>-0.1172641870784377</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4184,21 +4184,21 @@
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>7822</v>
+        <v>6914</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>倍利科</t>
+          <t>阜爾運通</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>305.3090005076195</v>
+        <v>306.6920692863387</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>810</v>
+        <v>120</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,13 +4209,13 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>35.55565953878212</v>
+        <v>20.28449379277681</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>11.08226315559839</v>
+        <v>41.58421132902605</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.6215765585742905</v>
+        <v>0.972105217746834</v>
       </c>
       <c r="K71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>-10.94084767010225</v>
+        <v>-0.3552812119583315</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6928</v>
+        <v>7822</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>攸泰科技</t>
+          <t>倍利科</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>304.2315362543339</v>
+        <v>305.3090005076195</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>47</v>
+        <v>810</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,13 +4262,13 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>44.30793203182547</v>
+        <v>35.55565953878212</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>11.4708668883819</v>
+        <v>11.08226315559839</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.6739201398007545</v>
+        <v>0.6215765585742905</v>
       </c>
       <c r="K72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.0391324205282467</v>
+        <v>-10.94084767010225</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>7818</v>
+        <v>6928</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>溢泰實業</t>
+          <t>攸泰科技</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>296.1294607314577</v>
+        <v>304.2315362543339</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>60.2</v>
+        <v>47</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,13 +4315,13 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>36.21766660272828</v>
+        <v>44.30793203182547</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>17.27913302428002</v>
+        <v>11.4708668883819</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.9465641799781266</v>
+        <v>0.6739201398007545</v>
       </c>
       <c r="K73" s="2" t="n">
         <v>0</v>
@@ -4333,31 +4333,31 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.104512823839149</v>
+        <v>-0.0391324205282467</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>7732</v>
+        <v>7818</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>金興精密</t>
+          <t>溢泰實業</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>294.0909513753142</v>
+        <v>296.1294607314577</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>34.15</v>
+        <v>60.2</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,13 +4368,13 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>48.80304886360786</v>
+        <v>36.21766660272828</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>6.386289730060585</v>
+        <v>17.27913302428002</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.6709254458059971</v>
+        <v>0.9465641799781266</v>
       </c>
       <c r="K74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-0.0376571274431666</v>
+        <v>0.104512823839149</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, williams_r_recovery</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6971</v>
+        <v>7732</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>惠民實業</t>
+          <t>金興精密</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>285.0843392339233</v>
+        <v>294.0909513753142</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>24.8</v>
+        <v>34.15</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>32.17330222361039</v>
+        <v>48.80304886360786</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>19.63726855468848</v>
+        <v>6.386289730060585</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.3076998818432453</v>
+        <v>0.6709254458059971</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.1304226130277933</v>
+        <v>-0.0376571274431666</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, williams_r_recovery</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>8034</v>
+        <v>6971</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>榮群</t>
+          <t>惠民實業</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>282.6080257536103</v>
+        <v>285.0843392339233</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>19.75</v>
+        <v>24.8</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,16 +4474,16 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>50.46592048848117</v>
+        <v>32.17330222361039</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>24.7335161831169</v>
+        <v>19.63726855468848</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.4325987396629936</v>
+        <v>0.3076998818432453</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.0604378432218399</v>
+        <v>-0.1304226130277933</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6890</v>
+        <v>8034</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>來億-KY</t>
+          <t>榮群</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>277.5916477634607</v>
+        <v>282.6080257536103</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>147.5</v>
+        <v>19.75</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,16 +4527,16 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>31.58711254838485</v>
+        <v>50.46592048848117</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>13.19672220048631</v>
+        <v>24.7335161831169</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.7680678623578753</v>
+        <v>0.4325987396629936</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-1.454082951010248</v>
+        <v>0.0604378432218399</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>7842</v>
+        <v>6890</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>天能綠電</t>
+          <t>來億-KY</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>274.3439374103478</v>
+        <v>277.5916477634607</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>99.5</v>
+        <v>147.5</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,13 +4580,13 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>53.20690060343706</v>
+        <v>31.58711254838485</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>18.98411789955327</v>
+        <v>13.19672220048631</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.2143184947223497</v>
+        <v>0.7680678623578753</v>
       </c>
       <c r="K78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.53229289226927</v>
+        <v>-1.454082951010248</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>8024</v>
+        <v>7842</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>佑華</t>
+          <t>天能綠電</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>274.1360497368806</v>
+        <v>274.3439374103478</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>12.6</v>
+        <v>99.5</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,16 +4633,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>33.55909479783199</v>
+        <v>53.20690060343706</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>13.6432416685908</v>
+        <v>18.98411789955327</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>1.000116054216913</v>
+        <v>0.2143184947223497</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.0216499926014919</v>
+        <v>-0.53229289226927</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>7730</v>
+        <v>8024</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>暉盛-創</t>
+          <t>佑華</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>273.3877339792451</v>
+        <v>274.1360497368806</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>168</v>
+        <v>12.6</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,16 +4686,16 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>46.30519953340434</v>
+        <v>33.55909479783199</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>19.08168632830779</v>
+        <v>13.6432416685908</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>0.2171099683274869</v>
+        <v>1.000116054216913</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>0</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-1.072462608010107</v>
+        <v>0.0216499926014919</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4714,21 +4714,21 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6996</v>
+        <v>7730</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>力領科技</t>
+          <t>暉盛-創</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>273.2220249164689</v>
+        <v>273.3877339792451</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>165.5</v>
+        <v>168</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,16 +4739,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>34.119900101488</v>
+        <v>46.30519953340434</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>19.00376661107582</v>
+        <v>19.08168632830779</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.3104662151319325</v>
+        <v>0.2171099683274869</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-1.693204093756913</v>
+        <v>-1.072462608010107</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6919</v>
+        <v>6996</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>康霈*</t>
+          <t>力領科技</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>269.3971948548853</v>
+        <v>273.2220249164689</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>79.3</v>
+        <v>165.5</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,16 +4792,16 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>30.92546103796682</v>
+        <v>34.119900101488</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>31.2680323125519</v>
+        <v>19.00376661107582</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.2471075859810984</v>
+        <v>0.3104662151319325</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L82" s="2" t="n">
         <v>0</v>
@@ -4810,31 +4810,31 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-1.574935119188787</v>
+        <v>-1.693204093756913</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6958</v>
+        <v>6919</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>日盛台駿</t>
+          <t>康霈*</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>260.9901578920601</v>
+        <v>269.3971948548853</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>17.35</v>
+        <v>79.3</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,13 +4845,13 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>46.26207614025344</v>
+        <v>30.92546103796682</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>18.18884773893128</v>
+        <v>31.2680323125519</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.7553283965688401</v>
+        <v>0.2471075859810984</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>0.0057942635466659</v>
+        <v>-1.574935119188787</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6994</v>
+        <v>6958</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>富威電力</t>
+          <t>日盛台駿</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>259.9913568026728</v>
+        <v>260.9901578920601</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>28</v>
+        <v>17.35</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>17.59911535004547</v>
+        <v>46.26207614025344</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>33.72112328920954</v>
+        <v>18.18884773893128</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>1.73690759559761</v>
+        <v>0.7553283965688401</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-0.5242145831627572</v>
+        <v>0.0057942635466659</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6903</v>
+        <v>6994</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>巨漢</t>
+          <t>富威電力</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>257.5224420810626</v>
+        <v>259.9913568026728</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>292</v>
+        <v>28</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>36.75575995294331</v>
+        <v>17.59911535004547</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>15.44303888124721</v>
+        <v>33.72112328920954</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>0.5286626540051423</v>
+        <v>1.73690759559761</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.5008595047765452</v>
+        <v>-0.5242145831627572</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6838</v>
+        <v>6903</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>台新藥</t>
+          <t>巨漢</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>256.1839690121539</v>
+        <v>257.5224420810626</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>23.4</v>
+        <v>292</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,13 +5004,13 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>46.99412207066126</v>
+        <v>36.75575995294331</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>18.94299438821536</v>
+        <v>15.44303888124721</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.5059630482493825</v>
+        <v>0.5286626540051423</v>
       </c>
       <c r="K86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.0348235988724468</v>
+        <v>-0.5008595047765452</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>7855</v>
+        <v>6838</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>和運租車</t>
+          <t>台新藥</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>256.0708547337415</v>
+        <v>256.1839690121539</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>42</v>
+        <v>23.4</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,13 +5057,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>17.50944841822879</v>
+        <v>46.99412207066126</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>55.0107391306835</v>
+        <v>18.94299438821536</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.4034349503077352</v>
+        <v>0.5059630482493825</v>
       </c>
       <c r="K87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>1.793366941552561</v>
+        <v>0.0348235988724468</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6909</v>
+        <v>7855</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>創控</t>
+          <t>和運租車</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>252.1289164459661</v>
+        <v>256.0708547337415</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>41.8</v>
+        <v>42</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>51.88509794960529</v>
+        <v>17.50944841822879</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>16.48110222702051</v>
+        <v>55.0107391306835</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>6.381145754612525</v>
+        <v>0.4034349503077352</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.394294324686796</v>
+        <v>1.793366941552561</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6921</v>
+        <v>6909</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>嘉雨思-創</t>
+          <t>創控</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>252.1205019035355</v>
+        <v>252.1289164459661</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>61</v>
+        <v>41.8</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,13 +5163,13 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>37.06295331593567</v>
+        <v>51.88509794960529</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>24.2439808783928</v>
+        <v>16.48110222702051</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.5761032377001959</v>
+        <v>6.381145754612525</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>-0.5258422005150231</v>
+        <v>0.394294324686796</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>7734</v>
+        <v>6921</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>印能科技</t>
+          <t>嘉雨思-創</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>251.1908252776356</v>
+        <v>252.1205019035355</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>2485</v>
+        <v>61</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,16 +5216,16 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>35.85522005787951</v>
+        <v>37.06295331593567</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>16.6815231573978</v>
+        <v>24.2439808783928</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>1.104178880396666</v>
+        <v>0.5761032377001959</v>
       </c>
       <c r="K90" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-25.50376149808173</v>
+        <v>-0.5258422005150231</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>7689</v>
+        <v>7734</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>大鵬科CLMX</t>
+          <t>印能科技</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>250.0835182549539</v>
+        <v>251.1908252776356</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>154.5</v>
+        <v>2485</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,16 +5269,16 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>23.6926031244015</v>
+        <v>35.85522005787951</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>28.01952776040346</v>
+        <v>16.6815231573978</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>0.2088857038212982</v>
+        <v>1.104178880396666</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.8702898905492473</v>
+        <v>-25.50376149808173</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>7721</v>
+        <v>7689</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>微程式</t>
+          <t>大鵬科CLMX</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>249.7577333608644</v>
+        <v>250.0835182549539</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>58.9</v>
+        <v>154.5</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,13 +5322,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>38.68150499622</v>
+        <v>23.6926031244015</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>12.75005445547253</v>
+        <v>28.01952776040346</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.6467749937198881</v>
+        <v>0.2088857038212982</v>
       </c>
       <c r="K92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.07804581972973</v>
+        <v>-0.8702898905492473</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6988</v>
+        <v>7721</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>威力暘-創</t>
+          <t>微程式</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>241.4515447140336</v>
+        <v>249.7577333608644</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>12</v>
+        <v>58.9</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>50.68844869852063</v>
+        <v>38.68150499622</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>9.166952375890194</v>
+        <v>12.75005445547253</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.5408828560417742</v>
+        <v>0.6467749937198881</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.07169021630995399</v>
+        <v>-0.07804581972973</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>7791</v>
+        <v>6988</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>皇家可口</t>
+          <t>威力暘-創</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>240.8608638886155</v>
+        <v>241.4515447140336</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>55.1</v>
+        <v>12</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,13 +5428,13 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>34.62946048365669</v>
+        <v>50.68844869852063</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>28.17656299678771</v>
+        <v>9.166952375890194</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.8576786958719921</v>
+        <v>0.5408828560417742</v>
       </c>
       <c r="K94" s="2" t="n">
         <v>0</v>
@@ -5446,31 +5446,31 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>0.0779568167547353</v>
+        <v>0.07169021630995399</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6873</v>
+        <v>7791</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>泓德能源</t>
+          <t>皇家可口</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>239.4902020854433</v>
+        <v>240.8608638886155</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>68</v>
+        <v>55.1</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,13 +5481,13 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>36.7515710338298</v>
+        <v>34.62946048365669</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>21.10224391229321</v>
+        <v>28.17656299678771</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>0.6805641196291149</v>
+        <v>0.8576786958719921</v>
       </c>
       <c r="K95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.4335879634011803</v>
+        <v>0.0779568167547353</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>7715</v>
+        <v>6873</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>裕山</t>
+          <t>泓德能源</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>238.7008649778368</v>
+        <v>239.4902020854433</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>27.65</v>
+        <v>68</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,13 +5534,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>30.26555605967869</v>
+        <v>36.7515710338298</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>29.02843905037317</v>
+        <v>21.10224391229321</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.9499490836587596</v>
+        <v>0.6805641196291149</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.1237366851209695</v>
+        <v>0.4335879634011803</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6934</v>
+        <v>7715</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>心誠鎂</t>
+          <t>裕山</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>236.2539889775098</v>
+        <v>238.7008649778368</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>73.09999999999999</v>
+        <v>27.65</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>45.66601937454406</v>
+        <v>30.26555605967869</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>16.71705088555356</v>
+        <v>29.02843905037317</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>1.516541845415546</v>
+        <v>0.9499490836587596</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>0.0341889816101924</v>
+        <v>-0.1237366851209695</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6899</v>
+        <v>6934</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>創為精密</t>
+          <t>心誠鎂</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>231.158199632834</v>
+        <v>236.2539889775098</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>49.1</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,16 +5640,16 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>32.93152132052107</v>
+        <v>45.66601937454406</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>21.48247074480715</v>
+        <v>16.71705088555356</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.5449773375227028</v>
+        <v>1.516541845415546</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>0.0471492823903085</v>
+        <v>0.0341889816101924</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6854</v>
+        <v>6899</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>錼創科技-KY創</t>
+          <t>創為精密</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>228.8437619750174</v>
+        <v>231.158199632834</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>89.2</v>
+        <v>49.1</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,16 +5693,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>41.08789796806827</v>
+        <v>32.93152132052107</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>16.85071191967015</v>
+        <v>21.48247074480715</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.3361439820762448</v>
+        <v>0.5449773375227028</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.041321000525806</v>
+        <v>0.0471492823903085</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>7805</v>
+        <v>6854</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>威聯通</t>
+          <t>錼創科技-KY創</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>227.1477473100026</v>
+        <v>228.8437619750174</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>497</v>
+        <v>89.2</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,16 +5746,16 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>30.71765341159879</v>
+        <v>41.08789796806827</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>38.39352751631359</v>
+        <v>16.85071191967015</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.3836715501153512</v>
+        <v>0.3361439820762448</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.8487118297632179</v>
+        <v>0.041321000525806</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>8032</v>
+        <v>7805</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>光菱</t>
+          <t>威聯通</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>221.4959457973783</v>
+        <v>227.1477473100026</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>34.55</v>
+        <v>497</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>33.96651110104042</v>
+        <v>30.71765341159879</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>23.68976839093457</v>
+        <v>38.39352751631359</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.5832017702779647</v>
+        <v>0.3836715501153512</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>1</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.0697335531861038</v>
+        <v>-0.8487118297632179</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5827,21 +5827,21 @@
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>7547</v>
+        <v>8032</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>碩網</t>
+          <t>光菱</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>215.7592373002831</v>
+        <v>221.4959457973783</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>49.5</v>
+        <v>34.55</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,16 +5852,16 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>42.52987320327906</v>
+        <v>33.96651110104042</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>10.6160934231438</v>
+        <v>23.68976839093457</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>3.741862932986997</v>
+        <v>0.5832017702779647</v>
       </c>
       <c r="K102" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.142270010379359</v>
+        <v>-0.0697335531861038</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>7722</v>
+        <v>7547</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>LINEPAY</t>
+          <t>碩網</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>211.1938583389341</v>
+        <v>215.7592373002831</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>265.5</v>
+        <v>49.5</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>39.11306938145643</v>
+        <v>42.52987320327906</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>11.9427580132916</v>
+        <v>10.6160934231438</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.8225335995590045</v>
+        <v>3.741862932986997</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-1.421255751427722</v>
+        <v>-0.142270010379359</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>volume_break, market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>7820</v>
+        <v>7722</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>立盈</t>
+          <t>LINEPAY</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>210.1715243730096</v>
+        <v>211.1938583389341</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>0</v>
+        <v>265.5</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>8.272403448339389</v>
+        <v>39.11306938145643</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>22.56729571075254</v>
+        <v>11.9427580132916</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.0190713889306224</v>
+        <v>0.8225335995590045</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-8.409378128073106</v>
+        <v>-1.421255751427722</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>7786</v>
+        <v>7820</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>東方風能</t>
+          <t>立盈</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>205.6309427274412</v>
+        <v>210.1715243730096</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>114</v>
+        <v>0</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>32.83760732768143</v>
+        <v>8.272403448339389</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>22.98263667223892</v>
+        <v>22.56729571075254</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.3470877829925837</v>
+        <v>0.0190713889306224</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.2105140074668918</v>
+        <v>-8.409378128073106</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6039,21 +6039,21 @@
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>8038</v>
+        <v>7786</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>長園科</t>
+          <t>東方風能</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>204.9208444368208</v>
+        <v>205.6309427274412</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>30</v>
+        <v>114</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,16 +6064,16 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>37.14496542860619</v>
+        <v>32.83760732768143</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>23.44036725715414</v>
+        <v>22.98263667223892</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.7325572519678538</v>
+        <v>0.3470877829925837</v>
       </c>
       <c r="K106" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L106" s="2" t="n">
         <v>0</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.0396945135440034</v>
+        <v>-0.2105140074668918</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6092,21 +6092,21 @@
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>7749</v>
+        <v>8038</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>意騰-KY</t>
+          <t>長園科</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>203.8829762090789</v>
+        <v>204.9208444368208</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>339</v>
+        <v>30</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,16 +6117,16 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>38.66972017536649</v>
+        <v>37.14496542860619</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>15.53854459684248</v>
+        <v>23.44036725715414</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.6438032459315109</v>
+        <v>0.7325572519678538</v>
       </c>
       <c r="K107" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-1.663657855194446</v>
+        <v>0.0396945135440034</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>6877</v>
+        <v>7749</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>鏵友益</t>
+          <t>意騰-KY</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>197.2283316990202</v>
+        <v>203.8829762090789</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>112</v>
+        <v>339</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>42.29969877658344</v>
+        <v>38.66972017536649</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>17.1731670464082</v>
+        <v>15.53854459684248</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.813918369623974</v>
+        <v>0.6438032459315109</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.137444643611079</v>
+        <v>-1.663657855194446</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>7736</v>
+        <v>6877</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>虎山</t>
+          <t>鏵友益</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>192.628609805093</v>
+        <v>197.2283316990202</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>68.40000000000001</v>
+        <v>112</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>39.80138972474536</v>
+        <v>42.29969877658344</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>13.56857040460083</v>
+        <v>17.1731670464082</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>3.011664206302296</v>
+        <v>0.813918369623974</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.0213527195563883</v>
+        <v>0.137444643611079</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>7760</v>
+        <v>7736</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>享溫馨</t>
+          <t>虎山</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>181.2051100658303</v>
+        <v>192.628609805093</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>33</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>47.38504705494583</v>
+        <v>39.80138972474536</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>10.22806157735667</v>
+        <v>13.56857040460083</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.6829767894406678</v>
+        <v>3.011664206302296</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.0006556998356470999</v>
+        <v>-0.0213527195563883</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6967</v>
+        <v>7760</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>汎瑋材料</t>
+          <t>享溫馨</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>179.5187217803398</v>
+        <v>181.2051100658303</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>64.7</v>
+        <v>33</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,16 +6329,16 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>32.88067886301019</v>
+        <v>47.38504705494583</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>13.50094647322398</v>
+        <v>10.22806157735667</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.8518721780339819</v>
+        <v>0.6829767894406678</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-0.891566876979125</v>
+        <v>-0.0006556998356470999</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>7740</v>
+        <v>6967</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>熙特爾-創</t>
+          <t>汎瑋材料</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>177.9341528734085</v>
+        <v>179.5187217803398</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>124</v>
+        <v>64.7</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,16 +6382,16 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>35.72809991857616</v>
+        <v>32.88067886301019</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>12.78301002284622</v>
+        <v>13.50094647322398</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>1.33538418446533</v>
+        <v>0.8518721780339819</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.0486628976496339</v>
+        <v>-0.891566876979125</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6947</v>
+        <v>7740</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>台鎔科技</t>
+          <t>熙特爾-創</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>175.74383726221</v>
+        <v>177.9341528734085</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>67.7</v>
+        <v>124</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>35.69304608475085</v>
+        <v>35.72809991857616</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>8.47713620730504</v>
+        <v>12.78301002284622</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.3802024703351337</v>
+        <v>1.33538418446533</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.20750553165617</v>
+        <v>-0.0486628976496339</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6463,21 +6463,21 @@
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>7821</v>
+        <v>6947</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>神數</t>
+          <t>台鎔科技</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>175.6028569801556</v>
+        <v>175.74383726221</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>38.7</v>
+        <v>67.7</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>39.44506939908622</v>
+        <v>35.69304608475085</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>12.57706363915899</v>
+        <v>8.47713620730504</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.9355007130684873</v>
+        <v>0.3802024703351337</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0332270870886963</v>
+        <v>0.20750553165617</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6516,21 +6516,21 @@
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>8011</v>
+        <v>7821</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>台通</t>
+          <t>神數</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>173.8267502629341</v>
+        <v>175.6028569801556</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>15.55</v>
+        <v>38.7</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>38.66154291637743</v>
+        <v>39.44506939908622</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>24.18117105859689</v>
+        <v>12.57706363915899</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.9332810706386314</v>
+        <v>0.9355007130684873</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.0076449771002017</v>
+        <v>0.0332270870886963</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6955</v>
+        <v>8011</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>邦睿生技-創</t>
+          <t>台通</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>171.2550292820653</v>
+        <v>173.8267502629341</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>0</v>
+        <v>15.55</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>22.53278947923667</v>
+        <v>38.66154291637743</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>11.12574580007753</v>
+        <v>24.18117105859689</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0</v>
+        <v>0.9332810706386314</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-7.16742832399968</v>
+        <v>-0.0076449771002017</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6869</v>
+        <v>6955</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>雲豹能源</t>
+          <t>邦睿生技-創</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>161.689842774302</v>
+        <v>171.2550292820653</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>63.5</v>
+        <v>0</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>39.2299702447481</v>
+        <v>22.53278947923667</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>10.99490220694683</v>
+        <v>11.12574580007753</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.4336026023404864</v>
+        <v>0</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.2320398205431681</v>
+        <v>-7.16742832399968</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6675,21 +6675,21 @@
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6862</v>
+        <v>6869</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>三集瑞-KY</t>
+          <t>雲豹能源</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>160.112679642896</v>
+        <v>161.689842774302</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>132</v>
+        <v>63.5</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,13 +6700,13 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>35.36439762334132</v>
+        <v>39.2299702447481</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>15.96282217591463</v>
+        <v>10.99490220694683</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.529181381189876</v>
+        <v>0.4336026023404864</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.07905960079519581</v>
+        <v>-0.2320398205431681</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6728,21 +6728,21 @@
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6923</v>
+        <v>6862</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>中台</t>
+          <t>三集瑞-KY</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>154.0842025456677</v>
+        <v>160.112679642896</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>75.7</v>
+        <v>132</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,13 +6753,13 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>45.9818398720866</v>
+        <v>35.36439762334132</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>9.254556709289142</v>
+        <v>15.96282217591463</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.8457489539037044</v>
+        <v>0.529181381189876</v>
       </c>
       <c r="K119" s="2" t="n">
         <v>0</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.0106743992918946</v>
+        <v>-0.07905960079519581</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6781,21 +6781,21 @@
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6901</v>
+        <v>6923</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>鑽石投資</t>
+          <t>中台</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>142.4080831060707</v>
+        <v>154.0842025456677</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>15.05</v>
+        <v>75.7</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,13 +6806,13 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>40.32503243534072</v>
+        <v>45.9818398720866</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>15.87302883533443</v>
+        <v>9.254556709289142</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.5851282801058767</v>
+        <v>0.8457489539037044</v>
       </c>
       <c r="K120" s="2" t="n">
         <v>0</v>
@@ -6824,31 +6824,31 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.0482278288346185</v>
+        <v>-0.0106743992918946</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>7827</v>
+        <v>6901</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>漢康-KY創</t>
+          <t>鑽石投資</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>135.8452633176145</v>
+        <v>142.4080831060707</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>152</v>
+        <v>15.05</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,13 +6859,13 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>44.89636025430854</v>
+        <v>40.32503243534072</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>12.76305347142746</v>
+        <v>15.87302883533443</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.3892898150914946</v>
+        <v>0.5851282801058767</v>
       </c>
       <c r="K121" s="2" t="n">
         <v>0</v>
@@ -6877,31 +6877,31 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.4569945794818254</v>
+        <v>-0.0482278288346185</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>6997</v>
+        <v>7827</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>博弘</t>
+          <t>漢康-KY創</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>132.7712310022288</v>
+        <v>135.8452633176145</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>0</v>
+        <v>152</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,13 +6912,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>40.78126991047967</v>
+        <v>44.89636025430854</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>9.942543545535711</v>
+        <v>12.76305347142746</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0</v>
+        <v>0.3892898150914946</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6930,31 +6930,31 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-7.26022101529083</v>
+        <v>-0.4569945794818254</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>7770</v>
+        <v>6997</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>君曜</t>
+          <t>博弘</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>128.3068689443578</v>
+        <v>132.7712310022288</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>36.5</v>
+        <v>0</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,16 +6965,16 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>50.33898219734937</v>
+        <v>40.78126991047967</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>4.854743606883081</v>
+        <v>9.942543545535711</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.3604983576477912</v>
+        <v>0</v>
       </c>
       <c r="K123" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L123" s="2" t="n">
         <v>0</v>
@@ -6983,31 +6983,31 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.06825394105139231</v>
+        <v>-7.26022101529083</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, above_ichimoku_cloud</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6855</v>
+        <v>7770</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>數泓科</t>
+          <t>君曜</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>127.9998062239094</v>
+        <v>128.3068689443578</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>113</v>
+        <v>36.5</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,16 +7018,16 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>51.78788592440718</v>
+        <v>50.33898219734937</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>8.187690797291845</v>
+        <v>4.854743606883081</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.3481341366076603</v>
+        <v>0.3604983576477912</v>
       </c>
       <c r="K124" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L124" s="2" t="n">
         <v>0</v>
@@ -7036,31 +7036,31 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>5.853299680401689</v>
+        <v>0.06825394105139231</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
+          <t>market_above_ma60, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>7753</v>
+        <v>6855</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>星亞</t>
+          <t>數泓科</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>120.8440539294933</v>
+        <v>127.9998062239094</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>36</v>
+        <v>113</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,13 +7071,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>35.32624359505456</v>
+        <v>51.78788592440718</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>9.703101695163266</v>
+        <v>8.187690797291845</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>0.824942210584359</v>
+        <v>0.3481341366076603</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7089,31 +7089,31 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>0.0507658218308455</v>
+        <v>5.853299680401689</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>7705</v>
+        <v>7753</v>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>三商餐飲</t>
+          <t>星亞</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>102.608196469947</v>
+        <v>120.8440539294933</v>
       </c>
       <c r="E126" s="2" t="n">
-        <v>29.85</v>
+        <v>36</v>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
@@ -7124,13 +7124,13 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>41.22788711590825</v>
+        <v>35.32624359505456</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>12.8754687745492</v>
+        <v>9.703101695163266</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>0.9338240324521406</v>
+        <v>0.824942210584359</v>
       </c>
       <c r="K126" s="2" t="n">
         <v>0</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.0364054867284159</v>
+        <v>0.0507658218308455</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7152,52 +7152,105 @@
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
+        <v>7705</v>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>三商餐飲</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D127" s="2" t="n">
+        <v>102.608196469947</v>
+      </c>
+      <c r="E127" s="2" t="n">
+        <v>29.85</v>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H127" s="2" t="n">
+        <v>41.22788711590825</v>
+      </c>
+      <c r="I127" s="2" t="n">
+        <v>12.8754687745492</v>
+      </c>
+      <c r="J127" s="2" t="n">
+        <v>0.9338240324521406</v>
+      </c>
+      <c r="K127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N127" s="2" t="n">
+        <v>-0.0364054867284159</v>
+      </c>
+      <c r="O127" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
         <v>7803</v>
       </c>
-      <c r="B127" s="2" t="inlineStr">
+      <c r="B128" s="2" t="inlineStr">
         <is>
           <t>雲象科技-創</t>
         </is>
       </c>
-      <c r="C127" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D127" s="2" t="n">
+      <c r="C128" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D128" s="2" t="n">
         <v>85.97519358543855</v>
       </c>
-      <c r="E127" s="2" t="n">
+      <c r="E128" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="F127" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14</t>
-        </is>
-      </c>
-      <c r="G127" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H127" s="2" t="n">
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H128" s="2" t="n">
         <v>40.59401897297612</v>
       </c>
-      <c r="I127" s="2" t="n">
+      <c r="I128" s="2" t="n">
         <v>9.488843124279478</v>
       </c>
-      <c r="J127" s="2" t="n">
+      <c r="J128" s="2" t="n">
         <v>1.464211800771767</v>
       </c>
-      <c r="K127" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L127" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M127" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N127" s="2" t="n">
+      <c r="K128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M128" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N128" s="2" t="n">
         <v>0.055376300181716</v>
       </c>
-      <c r="O127" s="2" t="inlineStr">
+      <c r="O128" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>